<commit_message>
No of Days Added Excel Added
</commit_message>
<xml_diff>
--- a/dataentry/uploaded_excel_files/cgl2019_new-website-sample-know-your-city-revised-data.xlsx
+++ b/dataentry/uploaded_excel_files/cgl2019_new-website-sample-know-your-city-revised-data.xlsx
@@ -1432,13 +1432,13 @@
     <t>PAPER III</t>
   </si>
   <si>
-    <t>CGL2019</t>
-  </si>
-  <si>
     <t>updated_on</t>
   </si>
   <si>
     <t>ipaddress</t>
+  </si>
+  <si>
+    <t>cgle2019</t>
   </si>
 </sst>
 </file>
@@ -1995,10 +1995,10 @@
         <v>50</v>
       </c>
       <c r="AZ1" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="BA1" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="BA1" s="3" t="s">
-        <v>474</v>
       </c>
       <c r="BB1" t="s">
         <v>51</v>
@@ -2149,7 +2149,7 @@
         <v>1</v>
       </c>
       <c r="BD2" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:58">
@@ -2289,7 +2289,7 @@
         <v>1</v>
       </c>
       <c r="BD3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="4" spans="1:58">
@@ -2429,7 +2429,7 @@
         <v>1</v>
       </c>
       <c r="BD4" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="5" spans="1:58">
@@ -2569,7 +2569,7 @@
         <v>1</v>
       </c>
       <c r="BD5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" spans="1:58">
@@ -2709,7 +2709,7 @@
         <v>1</v>
       </c>
       <c r="BD6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" spans="1:58">
@@ -2849,7 +2849,7 @@
         <v>1</v>
       </c>
       <c r="BD7" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" spans="1:58">
@@ -2989,7 +2989,7 @@
         <v>1</v>
       </c>
       <c r="BD8" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" spans="1:58">
@@ -3129,7 +3129,7 @@
         <v>1</v>
       </c>
       <c r="BD9" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="10" spans="1:58">
@@ -3269,7 +3269,7 @@
         <v>1</v>
       </c>
       <c r="BD10" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="11" spans="1:58">
@@ -3409,7 +3409,7 @@
         <v>1</v>
       </c>
       <c r="BD11" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" spans="1:58">
@@ -3549,7 +3549,7 @@
         <v>1</v>
       </c>
       <c r="BD12" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="13" spans="1:58">
@@ -3689,7 +3689,7 @@
         <v>1</v>
       </c>
       <c r="BD13" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="14" spans="1:58">
@@ -3829,7 +3829,7 @@
         <v>1</v>
       </c>
       <c r="BD14" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" spans="1:58">
@@ -3969,7 +3969,7 @@
         <v>1</v>
       </c>
       <c r="BD15" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="16" spans="1:58">
@@ -4109,7 +4109,7 @@
         <v>1</v>
       </c>
       <c r="BD16" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="17" spans="1:56">
@@ -4249,7 +4249,7 @@
         <v>1</v>
       </c>
       <c r="BD17" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="18" spans="1:56">
@@ -4389,7 +4389,7 @@
         <v>1</v>
       </c>
       <c r="BD18" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="19" spans="1:56">
@@ -4529,7 +4529,7 @@
         <v>1</v>
       </c>
       <c r="BD19" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="20" spans="1:56">
@@ -4669,7 +4669,7 @@
         <v>1</v>
       </c>
       <c r="BD20" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="21" spans="1:56">
@@ -4809,7 +4809,7 @@
         <v>1</v>
       </c>
       <c r="BD21" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="22" spans="1:56">
@@ -4949,7 +4949,7 @@
         <v>1</v>
       </c>
       <c r="BD22" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="23" spans="1:56">
@@ -5089,7 +5089,7 @@
         <v>1</v>
       </c>
       <c r="BD23" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="24" spans="1:56">
@@ -5229,7 +5229,7 @@
         <v>1</v>
       </c>
       <c r="BD24" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="25" spans="1:56">
@@ -5369,7 +5369,7 @@
         <v>1</v>
       </c>
       <c r="BD25" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="26" spans="1:56">
@@ -5509,7 +5509,7 @@
         <v>1</v>
       </c>
       <c r="BD26" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="27" spans="1:56">
@@ -5649,7 +5649,7 @@
         <v>1</v>
       </c>
       <c r="BD27" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="28" spans="1:56">
@@ -5789,7 +5789,7 @@
         <v>1</v>
       </c>
       <c r="BD28" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="29" spans="1:56">
@@ -5929,7 +5929,7 @@
         <v>1</v>
       </c>
       <c r="BD29" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="30" spans="1:56">
@@ -6069,7 +6069,7 @@
         <v>1</v>
       </c>
       <c r="BD30" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="31" spans="1:56">
@@ -6209,7 +6209,7 @@
         <v>1</v>
       </c>
       <c r="BD31" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="32" spans="1:56">
@@ -6349,7 +6349,7 @@
         <v>1</v>
       </c>
       <c r="BD32" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="33" spans="1:56">
@@ -6489,7 +6489,7 @@
         <v>1</v>
       </c>
       <c r="BD33" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="34" spans="1:56">
@@ -6629,7 +6629,7 @@
         <v>1</v>
       </c>
       <c r="BD34" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="35" spans="1:56">
@@ -6769,7 +6769,7 @@
         <v>1</v>
       </c>
       <c r="BD35" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="36" spans="1:56">
@@ -6909,7 +6909,7 @@
         <v>1</v>
       </c>
       <c r="BD36" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="37" spans="1:56">
@@ -7049,7 +7049,7 @@
         <v>1</v>
       </c>
       <c r="BD37" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="38" spans="1:56">
@@ -7189,7 +7189,7 @@
         <v>1</v>
       </c>
       <c r="BD38" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="39" spans="1:56">
@@ -7329,7 +7329,7 @@
         <v>1</v>
       </c>
       <c r="BD39" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="40" spans="1:56">
@@ -7469,7 +7469,7 @@
         <v>1</v>
       </c>
       <c r="BD40" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="41" spans="1:56">
@@ -7609,7 +7609,7 @@
         <v>1</v>
       </c>
       <c r="BD41" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="42" spans="1:56">
@@ -7749,7 +7749,7 @@
         <v>1</v>
       </c>
       <c r="BD42" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="43" spans="1:56">
@@ -7889,7 +7889,7 @@
         <v>1</v>
       </c>
       <c r="BD43" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="44" spans="1:56">
@@ -8029,7 +8029,7 @@
         <v>1</v>
       </c>
       <c r="BD44" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="45" spans="1:56">
@@ -8169,7 +8169,7 @@
         <v>1</v>
       </c>
       <c r="BD45" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="46" spans="1:56">
@@ -8309,7 +8309,7 @@
         <v>1</v>
       </c>
       <c r="BD46" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="47" spans="1:56">
@@ -8449,7 +8449,7 @@
         <v>1</v>
       </c>
       <c r="BD47" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="48" spans="1:56">
@@ -8589,7 +8589,7 @@
         <v>1</v>
       </c>
       <c r="BD48" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="49" spans="1:56">
@@ -8729,7 +8729,7 @@
         <v>1</v>
       </c>
       <c r="BD49" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="50" spans="1:56">
@@ -8869,7 +8869,7 @@
         <v>1</v>
       </c>
       <c r="BD50" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="51" spans="1:56">
@@ -9009,7 +9009,7 @@
         <v>1</v>
       </c>
       <c r="BD51" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="52" spans="1:56">
@@ -9149,7 +9149,7 @@
         <v>1</v>
       </c>
       <c r="BD52" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="53" spans="1:56">
@@ -9289,7 +9289,7 @@
         <v>1</v>
       </c>
       <c r="BD53" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="54" spans="1:56">
@@ -9429,7 +9429,7 @@
         <v>1</v>
       </c>
       <c r="BD54" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="55" spans="1:56">
@@ -9569,7 +9569,7 @@
         <v>1</v>
       </c>
       <c r="BD55" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="56" spans="1:56">
@@ -9709,7 +9709,7 @@
         <v>1</v>
       </c>
       <c r="BD56" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="57" spans="1:56">
@@ -9849,7 +9849,7 @@
         <v>1</v>
       </c>
       <c r="BD57" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="58" spans="1:56">
@@ -9989,7 +9989,7 @@
         <v>1</v>
       </c>
       <c r="BD58" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="59" spans="1:56">
@@ -10129,7 +10129,7 @@
         <v>1</v>
       </c>
       <c r="BD59" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="60" spans="1:56">
@@ -10269,7 +10269,7 @@
         <v>1</v>
       </c>
       <c r="BD60" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="61" spans="1:56">
@@ -10409,7 +10409,7 @@
         <v>1</v>
       </c>
       <c r="BD61" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="62" spans="1:56">
@@ -10549,7 +10549,7 @@
         <v>1</v>
       </c>
       <c r="BD62" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="63" spans="1:56">
@@ -10689,7 +10689,7 @@
         <v>1</v>
       </c>
       <c r="BD63" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="64" spans="1:56">
@@ -10829,7 +10829,7 @@
         <v>1</v>
       </c>
       <c r="BD64" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="65" spans="1:56">
@@ -10969,7 +10969,7 @@
         <v>1</v>
       </c>
       <c r="BD65" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="66" spans="1:56">
@@ -11109,7 +11109,7 @@
         <v>1</v>
       </c>
       <c r="BD66" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="67" spans="1:56">
@@ -11249,7 +11249,7 @@
         <v>1</v>
       </c>
       <c r="BD67" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="68" spans="1:56">
@@ -11389,7 +11389,7 @@
         <v>1</v>
       </c>
       <c r="BD68" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="69" spans="1:56">
@@ -11529,7 +11529,7 @@
         <v>1</v>
       </c>
       <c r="BD69" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="70" spans="1:56">
@@ -11669,7 +11669,7 @@
         <v>1</v>
       </c>
       <c r="BD70" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="71" spans="1:56">
@@ -11809,7 +11809,7 @@
         <v>1</v>
       </c>
       <c r="BD71" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="72" spans="1:56">
@@ -11949,7 +11949,7 @@
         <v>1</v>
       </c>
       <c r="BD72" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="73" spans="1:56">
@@ -12089,7 +12089,7 @@
         <v>1</v>
       </c>
       <c r="BD73" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="74" spans="1:56">
@@ -12229,7 +12229,7 @@
         <v>1</v>
       </c>
       <c r="BD74" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="75" spans="1:56">
@@ -12369,7 +12369,7 @@
         <v>1</v>
       </c>
       <c r="BD75" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="76" spans="1:56">
@@ -12509,7 +12509,7 @@
         <v>1</v>
       </c>
       <c r="BD76" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="77" spans="1:56">
@@ -12649,7 +12649,7 @@
         <v>1</v>
       </c>
       <c r="BD77" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="78" spans="1:56">
@@ -12789,7 +12789,7 @@
         <v>1</v>
       </c>
       <c r="BD78" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="79" spans="1:56">
@@ -12929,7 +12929,7 @@
         <v>1</v>
       </c>
       <c r="BD79" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="80" spans="1:56">
@@ -13069,7 +13069,7 @@
         <v>1</v>
       </c>
       <c r="BD80" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="81" spans="1:56">
@@ -13209,7 +13209,7 @@
         <v>1</v>
       </c>
       <c r="BD81" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="82" spans="1:56">
@@ -13349,7 +13349,7 @@
         <v>1</v>
       </c>
       <c r="BD82" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="83" spans="1:56">
@@ -13489,7 +13489,7 @@
         <v>1</v>
       </c>
       <c r="BD83" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="84" spans="1:56">
@@ -13629,7 +13629,7 @@
         <v>1</v>
       </c>
       <c r="BD84" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="85" spans="1:56">
@@ -13769,7 +13769,7 @@
         <v>1</v>
       </c>
       <c r="BD85" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="86" spans="1:56">
@@ -13909,7 +13909,7 @@
         <v>1</v>
       </c>
       <c r="BD86" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="87" spans="1:56">
@@ -14049,7 +14049,7 @@
         <v>1</v>
       </c>
       <c r="BD87" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="88" spans="1:56">
@@ -14189,7 +14189,7 @@
         <v>1</v>
       </c>
       <c r="BD88" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="89" spans="1:56">
@@ -14329,7 +14329,7 @@
         <v>1</v>
       </c>
       <c r="BD89" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="90" spans="1:56">
@@ -14469,7 +14469,7 @@
         <v>1</v>
       </c>
       <c r="BD90" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="91" spans="1:56">
@@ -14609,7 +14609,7 @@
         <v>1</v>
       </c>
       <c r="BD91" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="92" spans="1:56">
@@ -14749,7 +14749,7 @@
         <v>1</v>
       </c>
       <c r="BD92" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="93" spans="1:56">
@@ -14889,7 +14889,7 @@
         <v>1</v>
       </c>
       <c r="BD93" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="94" spans="1:56">
@@ -15029,7 +15029,7 @@
         <v>1</v>
       </c>
       <c r="BD94" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="95" spans="1:56">
@@ -15169,7 +15169,7 @@
         <v>1</v>
       </c>
       <c r="BD95" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="96" spans="1:56">
@@ -15309,7 +15309,7 @@
         <v>1</v>
       </c>
       <c r="BD96" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="97" spans="1:56">
@@ -15449,7 +15449,7 @@
         <v>1</v>
       </c>
       <c r="BD97" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="98" spans="1:56">
@@ -15589,7 +15589,7 @@
         <v>1</v>
       </c>
       <c r="BD98" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="99" spans="1:56">
@@ -15729,7 +15729,7 @@
         <v>1</v>
       </c>
       <c r="BD99" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="100" spans="1:56">
@@ -15869,7 +15869,7 @@
         <v>1</v>
       </c>
       <c r="BD100" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="101" spans="1:56">
@@ -16009,7 +16009,7 @@
         <v>1</v>
       </c>
       <c r="BD101" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>